<commit_message>
feat: implement creative view enhancements, Akinator fix, and full Docker containerization
</commit_message>
<xml_diff>
--- a/01 - Atrib Atual No Cor.xlsx
+++ b/01 - Atrib Atual No Cor.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Associação\Atribuições Cargos\Tabelas de Atribuições\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maiap\OneDrive\Desktop\Desenvolvimento\Estudo_Atribuicoes_PCSP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A81E5DAB-622A-46E9-84CA-23DDADA71B11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0BD55DC-5817-489A-AF5B-B8DFC12D0E2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{9E2F6A9B-94A3-41DD-92E9-2C4405031CDE}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{9E2F6A9B-94A3-41DD-92E9-2C4405031CDE}"/>
   </bookViews>
   <sheets>
     <sheet name="Carreiras e Atribuicoes sem cor" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
   <si>
     <t>mediar conflitos</t>
   </si>
@@ -230,36 +230,6 @@
   </si>
   <si>
     <t>Atendente de Necrotério Policial</t>
-  </si>
-  <si>
-    <t>portar arma, distintivo e algemas</t>
-  </si>
-  <si>
-    <t>atender sempre, com urbanidade e eficiência, o público em geral, pessoalmente ou por telefone</t>
-  </si>
-  <si>
-    <t>elaborar, sob orientação da Autoridade Policial, registro de ocorrência</t>
-  </si>
-  <si>
-    <t>conduzir viatura policial</t>
-  </si>
-  <si>
-    <t>cumprir diligência e/ou requisição determinada pela Autoridade Policial, elaborando relatório respectivo</t>
-  </si>
-  <si>
-    <t>proceder à abordagem de pessoas suspeitas da prática de ilícitos, realizando busca pessoal quando necessário</t>
-  </si>
-  <si>
-    <t>identificar pessoas, inclusive por meio digital, nas hipóteses em que tal providência se faça necessária</t>
-  </si>
-  <si>
-    <t>conduzir e apresentar pessoas legalmente presas à Autoridade Policial competente ou onde for por ela determinado</t>
-  </si>
-  <si>
-    <t>auxiliar a Autoridade Policial na formalização de atos de polícia judiciária</t>
-  </si>
-  <si>
-    <t>operar os sistemas de comunicação e de dados da Polícia Civil</t>
   </si>
   <si>
     <t>gestão de polícia judiciária</t>
@@ -1186,62 +1156,52 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61E66DEB-712A-465C-882E-F5424BC162B6}">
-  <dimension ref="A1:BU15"/>
+  <dimension ref="A1:BK15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="29.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="29.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="30.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="30.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="27.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="31.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="26.109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.44140625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="8" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="30" max="31" width="8.77734375" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="37" max="38" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="43" max="46" width="8.21875" bestFit="1" customWidth="1"/>
-    <col min="47" max="48" width="8.77734375" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="8.77734375" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="8.77734375" bestFit="1" customWidth="1"/>
-    <col min="55" max="56" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="8.77734375" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="8" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="69" max="71" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="8" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="25" max="26" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="27" max="28" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="33" max="36" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="37" max="38" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="45" max="46" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="8" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="59" max="61" width="8.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:73" s="1" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:63" s="1" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>70</v>
@@ -1253,214 +1213,184 @@
         <v>72</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="F1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="M1" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="N1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="S1" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>4</v>
-      </c>
       <c r="T1" s="3" t="s">
-        <v>86</v>
+        <v>12</v>
       </c>
       <c r="U1" s="3" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="V1" s="3" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="W1" s="3" t="s">
-        <v>84</v>
+        <v>15</v>
       </c>
       <c r="X1" s="3" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="Y1" s="3" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="Z1" s="3" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="AA1" s="3" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="AB1" s="3" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="AC1" s="3" t="s">
-        <v>85</v>
+        <v>21</v>
       </c>
       <c r="AD1" s="3" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="AE1" s="3" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="AF1" s="3" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="AG1" s="3" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="AH1" s="3" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="AI1" s="3" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="AJ1" s="3" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="AK1" s="3" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="AL1" s="3" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="AM1" s="3" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="AN1" s="3" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="AO1" s="3" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="AP1" s="3" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="AQ1" s="3" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="AR1" s="3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="AS1" s="3" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="AT1" s="3" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="AU1" s="3" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="AV1" s="3" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="AW1" s="3" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="AX1" s="3" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="AY1" s="3" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="AZ1" s="3" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="BA1" s="3" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="BB1" s="3" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="BC1" s="3" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="BD1" s="3" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="BE1" s="3" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="BF1" s="3" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="BG1" s="3" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="BH1" s="3" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="BI1" s="3" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="BJ1" s="3" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="BK1" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="BL1" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="BM1" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="BN1" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="BO1" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="BP1" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="BQ1" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="BR1" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="BS1" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="BT1" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="BU1" s="3" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:73" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>56</v>
       </c>
@@ -1477,34 +1407,34 @@
         <v>1</v>
       </c>
       <c r="F2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P2" s="5">
         <v>0</v>
@@ -1650,52 +1580,22 @@
       <c r="BK2" s="5">
         <v>0</v>
       </c>
-      <c r="BL2" s="5">
-        <v>0</v>
-      </c>
-      <c r="BM2" s="5">
-        <v>0</v>
-      </c>
-      <c r="BN2" s="5">
-        <v>0</v>
-      </c>
-      <c r="BO2" s="5">
-        <v>0</v>
-      </c>
-      <c r="BP2" s="5">
-        <v>0</v>
-      </c>
-      <c r="BQ2" s="5">
-        <v>0</v>
-      </c>
-      <c r="BR2" s="5">
-        <v>0</v>
-      </c>
-      <c r="BS2" s="5">
-        <v>0</v>
-      </c>
-      <c r="BT2" s="5">
-        <v>0</v>
-      </c>
-      <c r="BU2" s="5">
-        <v>0</v>
-      </c>
     </row>
-    <row r="3" spans="1:73" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>57</v>
       </c>
       <c r="B3" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" s="5">
         <v>1</v>
@@ -1710,10 +1610,10 @@
         <v>1</v>
       </c>
       <c r="J3" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K3" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L3" s="5">
         <v>0</v>
@@ -1728,16 +1628,16 @@
         <v>0</v>
       </c>
       <c r="P3" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q3" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R3" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S3" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T3" s="5">
         <v>0</v>
@@ -1871,64 +1771,34 @@
       <c r="BK3" s="5">
         <v>0</v>
       </c>
-      <c r="BL3" s="5">
-        <v>0</v>
-      </c>
-      <c r="BM3" s="5">
-        <v>0</v>
-      </c>
-      <c r="BN3" s="5">
-        <v>0</v>
-      </c>
-      <c r="BO3" s="5">
-        <v>0</v>
-      </c>
-      <c r="BP3" s="5">
-        <v>0</v>
-      </c>
-      <c r="BQ3" s="5">
-        <v>0</v>
-      </c>
-      <c r="BR3" s="5">
-        <v>0</v>
-      </c>
-      <c r="BS3" s="5">
-        <v>0</v>
-      </c>
-      <c r="BT3" s="5">
-        <v>0</v>
-      </c>
-      <c r="BU3" s="5">
-        <v>0</v>
-      </c>
     </row>
-    <row r="4" spans="1:73" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>58</v>
       </c>
       <c r="B4" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C4" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I4" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" s="5">
         <v>1</v>
@@ -1937,19 +1807,19 @@
         <v>1</v>
       </c>
       <c r="L4" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M4" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N4" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O4" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P4" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q4" s="5">
         <v>0</v>
@@ -1961,25 +1831,25 @@
         <v>0</v>
       </c>
       <c r="T4" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U4" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V4" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W4" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X4" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y4" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z4" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA4" s="5">
         <v>0</v>
@@ -2092,70 +1962,40 @@
       <c r="BK4" s="5">
         <v>0</v>
       </c>
-      <c r="BL4" s="5">
-        <v>0</v>
-      </c>
-      <c r="BM4" s="5">
-        <v>0</v>
-      </c>
-      <c r="BN4" s="5">
-        <v>0</v>
-      </c>
-      <c r="BO4" s="5">
-        <v>0</v>
-      </c>
-      <c r="BP4" s="5">
-        <v>0</v>
-      </c>
-      <c r="BQ4" s="5">
-        <v>0</v>
-      </c>
-      <c r="BR4" s="5">
-        <v>0</v>
-      </c>
-      <c r="BS4" s="5">
-        <v>0</v>
-      </c>
-      <c r="BT4" s="5">
-        <v>0</v>
-      </c>
-      <c r="BU4" s="5">
-        <v>0</v>
-      </c>
     </row>
-    <row r="5" spans="1:73" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>59</v>
       </c>
       <c r="B5" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C5" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H5" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I5" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K5" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L5" s="5">
         <v>0</v>
@@ -2173,34 +2013,34 @@
         <v>0</v>
       </c>
       <c r="Q5" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R5" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S5" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T5" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U5" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V5" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W5" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X5" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y5" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z5" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA5" s="5">
         <v>1</v>
@@ -2218,34 +2058,34 @@
         <v>1</v>
       </c>
       <c r="AF5" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG5" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH5" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI5" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ5" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AK5" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AL5" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AM5" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN5" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO5" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP5" s="5">
         <v>0</v>
@@ -2313,70 +2153,40 @@
       <c r="BK5" s="5">
         <v>0</v>
       </c>
-      <c r="BL5" s="5">
-        <v>0</v>
-      </c>
-      <c r="BM5" s="5">
-        <v>0</v>
-      </c>
-      <c r="BN5" s="5">
-        <v>0</v>
-      </c>
-      <c r="BO5" s="5">
-        <v>0</v>
-      </c>
-      <c r="BP5" s="5">
-        <v>0</v>
-      </c>
-      <c r="BQ5" s="5">
-        <v>0</v>
-      </c>
-      <c r="BR5" s="5">
-        <v>0</v>
-      </c>
-      <c r="BS5" s="5">
-        <v>0</v>
-      </c>
-      <c r="BT5" s="5">
-        <v>0</v>
-      </c>
-      <c r="BU5" s="5">
-        <v>0</v>
-      </c>
     </row>
-    <row r="6" spans="1:73" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>60</v>
       </c>
       <c r="B6" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C6" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H6" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I6" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J6" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K6" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L6" s="5">
         <v>0</v>
@@ -2406,13 +2216,13 @@
         <v>0</v>
       </c>
       <c r="U6" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V6" s="5">
         <v>0</v>
       </c>
       <c r="W6" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X6" s="5">
         <v>0</v>
@@ -2427,7 +2237,7 @@
         <v>0</v>
       </c>
       <c r="AB6" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC6" s="5">
         <v>0</v>
@@ -2436,19 +2246,19 @@
         <v>0</v>
       </c>
       <c r="AE6" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF6" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG6" s="5">
         <v>1</v>
       </c>
       <c r="AH6" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI6" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ6" s="5">
         <v>0</v>
@@ -2457,7 +2267,7 @@
         <v>0</v>
       </c>
       <c r="AL6" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AM6" s="5">
         <v>0</v>
@@ -2469,16 +2279,16 @@
         <v>0</v>
       </c>
       <c r="AP6" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ6" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR6" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS6" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT6" s="5">
         <v>0</v>
@@ -2534,70 +2344,40 @@
       <c r="BK6" s="5">
         <v>0</v>
       </c>
-      <c r="BL6" s="5">
-        <v>0</v>
-      </c>
-      <c r="BM6" s="5">
-        <v>0</v>
-      </c>
-      <c r="BN6" s="5">
-        <v>0</v>
-      </c>
-      <c r="BO6" s="5">
-        <v>0</v>
-      </c>
-      <c r="BP6" s="5">
-        <v>0</v>
-      </c>
-      <c r="BQ6" s="5">
-        <v>0</v>
-      </c>
-      <c r="BR6" s="5">
-        <v>0</v>
-      </c>
-      <c r="BS6" s="5">
-        <v>0</v>
-      </c>
-      <c r="BT6" s="5">
-        <v>0</v>
-      </c>
-      <c r="BU6" s="5">
-        <v>0</v>
-      </c>
     </row>
-    <row r="7" spans="1:73" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>61</v>
       </c>
       <c r="B7" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C7" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H7" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I7" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J7" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K7" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L7" s="5">
         <v>0</v>
@@ -2621,7 +2401,7 @@
         <v>0</v>
       </c>
       <c r="S7" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T7" s="5">
         <v>0</v>
@@ -2672,28 +2452,28 @@
         <v>0</v>
       </c>
       <c r="AJ7" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AK7" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL7" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM7" s="5">
         <v>1</v>
       </c>
       <c r="AN7" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO7" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP7" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ7" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR7" s="5">
         <v>0</v>
@@ -2702,28 +2482,28 @@
         <v>0</v>
       </c>
       <c r="AT7" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU7" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV7" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AW7" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX7" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AY7" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AZ7" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BA7" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BB7" s="5">
         <v>0</v>
@@ -2755,70 +2535,40 @@
       <c r="BK7" s="5">
         <v>0</v>
       </c>
-      <c r="BL7" s="5">
-        <v>0</v>
-      </c>
-      <c r="BM7" s="5">
-        <v>0</v>
-      </c>
-      <c r="BN7" s="5">
-        <v>0</v>
-      </c>
-      <c r="BO7" s="5">
-        <v>0</v>
-      </c>
-      <c r="BP7" s="5">
-        <v>0</v>
-      </c>
-      <c r="BQ7" s="5">
-        <v>0</v>
-      </c>
-      <c r="BR7" s="5">
-        <v>0</v>
-      </c>
-      <c r="BS7" s="5">
-        <v>0</v>
-      </c>
-      <c r="BT7" s="5">
-        <v>0</v>
-      </c>
-      <c r="BU7" s="5">
-        <v>0</v>
-      </c>
     </row>
-    <row r="8" spans="1:73" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>62</v>
       </c>
       <c r="B8" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C8" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H8" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J8" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L8" s="5">
         <v>0</v>
@@ -2842,7 +2592,7 @@
         <v>0</v>
       </c>
       <c r="S8" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T8" s="5">
         <v>0</v>
@@ -2902,7 +2652,7 @@
         <v>0</v>
       </c>
       <c r="AM8" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN8" s="5">
         <v>0</v>
@@ -2917,13 +2667,13 @@
         <v>0</v>
       </c>
       <c r="AR8" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS8" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT8" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU8" s="5">
         <v>0</v>
@@ -2947,13 +2697,13 @@
         <v>0</v>
       </c>
       <c r="BB8" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BC8" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BD8" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BE8" s="5">
         <v>0</v>
@@ -2976,70 +2726,40 @@
       <c r="BK8" s="5">
         <v>0</v>
       </c>
-      <c r="BL8" s="5">
-        <v>0</v>
-      </c>
-      <c r="BM8" s="5">
-        <v>0</v>
-      </c>
-      <c r="BN8" s="5">
-        <v>0</v>
-      </c>
-      <c r="BO8" s="5">
-        <v>0</v>
-      </c>
-      <c r="BP8" s="5">
-        <v>0</v>
-      </c>
-      <c r="BQ8" s="5">
-        <v>0</v>
-      </c>
-      <c r="BR8" s="5">
-        <v>0</v>
-      </c>
-      <c r="BS8" s="5">
-        <v>0</v>
-      </c>
-      <c r="BT8" s="5">
-        <v>0</v>
-      </c>
-      <c r="BU8" s="5">
-        <v>0</v>
-      </c>
     </row>
-    <row r="9" spans="1:73" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>63</v>
       </c>
       <c r="B9" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C9" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D9" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H9" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I9" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L9" s="5">
         <v>0</v>
@@ -3197,70 +2917,40 @@
       <c r="BK9" s="5">
         <v>0</v>
       </c>
-      <c r="BL9" s="5">
-        <v>0</v>
-      </c>
-      <c r="BM9" s="5">
-        <v>0</v>
-      </c>
-      <c r="BN9" s="5">
-        <v>0</v>
-      </c>
-      <c r="BO9" s="5">
-        <v>0</v>
-      </c>
-      <c r="BP9" s="5">
-        <v>0</v>
-      </c>
-      <c r="BQ9" s="5">
-        <v>0</v>
-      </c>
-      <c r="BR9" s="5">
-        <v>0</v>
-      </c>
-      <c r="BS9" s="5">
-        <v>0</v>
-      </c>
-      <c r="BT9" s="5">
-        <v>0</v>
-      </c>
-      <c r="BU9" s="5">
-        <v>0</v>
-      </c>
     </row>
-    <row r="10" spans="1:73" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>64</v>
       </c>
       <c r="B10" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C10" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D10" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H10" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I10" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J10" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L10" s="5">
         <v>0</v>
@@ -3418,70 +3108,40 @@
       <c r="BK10" s="5">
         <v>0</v>
       </c>
-      <c r="BL10" s="5">
-        <v>0</v>
-      </c>
-      <c r="BM10" s="5">
-        <v>0</v>
-      </c>
-      <c r="BN10" s="5">
-        <v>0</v>
-      </c>
-      <c r="BO10" s="5">
-        <v>0</v>
-      </c>
-      <c r="BP10" s="5">
-        <v>0</v>
-      </c>
-      <c r="BQ10" s="5">
-        <v>0</v>
-      </c>
-      <c r="BR10" s="5">
-        <v>0</v>
-      </c>
-      <c r="BS10" s="5">
-        <v>0</v>
-      </c>
-      <c r="BT10" s="5">
-        <v>0</v>
-      </c>
-      <c r="BU10" s="5">
-        <v>0</v>
-      </c>
     </row>
-    <row r="11" spans="1:73" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>65</v>
       </c>
       <c r="B11" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C11" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D11" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E11" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F11" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I11" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J11" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L11" s="5">
         <v>0</v>
@@ -3639,70 +3299,40 @@
       <c r="BK11" s="5">
         <v>0</v>
       </c>
-      <c r="BL11" s="5">
-        <v>0</v>
-      </c>
-      <c r="BM11" s="5">
-        <v>0</v>
-      </c>
-      <c r="BN11" s="5">
-        <v>0</v>
-      </c>
-      <c r="BO11" s="5">
-        <v>0</v>
-      </c>
-      <c r="BP11" s="5">
-        <v>0</v>
-      </c>
-      <c r="BQ11" s="5">
-        <v>0</v>
-      </c>
-      <c r="BR11" s="5">
-        <v>0</v>
-      </c>
-      <c r="BS11" s="5">
-        <v>0</v>
-      </c>
-      <c r="BT11" s="5">
-        <v>0</v>
-      </c>
-      <c r="BU11" s="5">
-        <v>0</v>
-      </c>
     </row>
-    <row r="12" spans="1:73" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>66</v>
       </c>
       <c r="B12" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C12" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D12" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H12" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I12" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J12" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K12" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L12" s="5">
         <v>0</v>
@@ -3738,7 +3368,7 @@
         <v>0</v>
       </c>
       <c r="W12" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X12" s="5">
         <v>0</v>
@@ -3768,7 +3398,7 @@
         <v>0</v>
       </c>
       <c r="AG12" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH12" s="5">
         <v>0</v>
@@ -3810,19 +3440,19 @@
         <v>0</v>
       </c>
       <c r="AU12" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV12" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW12" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX12" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY12" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AZ12" s="5">
         <v>0</v>
@@ -3840,19 +3470,19 @@
         <v>0</v>
       </c>
       <c r="BE12" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BF12" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BG12" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BH12" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BI12" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BJ12" s="5">
         <v>0</v>
@@ -3860,76 +3490,46 @@
       <c r="BK12" s="5">
         <v>0</v>
       </c>
-      <c r="BL12" s="5">
-        <v>0</v>
-      </c>
-      <c r="BM12" s="5">
-        <v>0</v>
-      </c>
-      <c r="BN12" s="5">
-        <v>0</v>
-      </c>
-      <c r="BO12" s="5">
-        <v>0</v>
-      </c>
-      <c r="BP12" s="5">
-        <v>0</v>
-      </c>
-      <c r="BQ12" s="5">
-        <v>0</v>
-      </c>
-      <c r="BR12" s="5">
-        <v>0</v>
-      </c>
-      <c r="BS12" s="5">
-        <v>0</v>
-      </c>
-      <c r="BT12" s="5">
-        <v>0</v>
-      </c>
-      <c r="BU12" s="5">
-        <v>0</v>
-      </c>
     </row>
-    <row r="13" spans="1:73" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>67</v>
       </c>
       <c r="B13" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C13" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D13" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H13" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J13" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K13" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L13" s="5">
         <v>0</v>
       </c>
       <c r="M13" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N13" s="5">
         <v>0</v>
@@ -3977,7 +3577,7 @@
         <v>0</v>
       </c>
       <c r="AC13" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD13" s="5">
         <v>0</v>
@@ -3989,7 +3589,7 @@
         <v>0</v>
       </c>
       <c r="AG13" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH13" s="5">
         <v>0</v>
@@ -4007,7 +3607,7 @@
         <v>0</v>
       </c>
       <c r="AM13" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN13" s="5">
         <v>0</v>
@@ -4034,7 +3634,7 @@
         <v>0</v>
       </c>
       <c r="AV13" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW13" s="5">
         <v>0</v>
@@ -4046,10 +3646,10 @@
         <v>0</v>
       </c>
       <c r="AZ13" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BA13" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BB13" s="5">
         <v>0</v>
@@ -4064,7 +3664,7 @@
         <v>0</v>
       </c>
       <c r="BF13" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BG13" s="5">
         <v>0</v>
@@ -4076,75 +3676,45 @@
         <v>0</v>
       </c>
       <c r="BJ13" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BK13" s="5">
-        <v>1</v>
-      </c>
-      <c r="BL13" s="5">
-        <v>0</v>
-      </c>
-      <c r="BM13" s="5">
-        <v>0</v>
-      </c>
-      <c r="BN13" s="5">
-        <v>0</v>
-      </c>
-      <c r="BO13" s="5">
-        <v>0</v>
-      </c>
-      <c r="BP13" s="5">
-        <v>0</v>
-      </c>
-      <c r="BQ13" s="5">
-        <v>0</v>
-      </c>
-      <c r="BR13" s="5">
-        <v>0</v>
-      </c>
-      <c r="BS13" s="5">
-        <v>0</v>
-      </c>
-      <c r="BT13" s="5">
-        <v>0</v>
-      </c>
-      <c r="BU13" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:73" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>68</v>
       </c>
       <c r="B14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L14" s="5">
         <v>0</v>
@@ -4195,7 +3765,7 @@
         <v>0</v>
       </c>
       <c r="AB14" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC14" s="5">
         <v>0</v>
@@ -4225,7 +3795,7 @@
         <v>0</v>
       </c>
       <c r="AL14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AM14" s="5">
         <v>0</v>
@@ -4273,16 +3843,16 @@
         <v>0</v>
       </c>
       <c r="BB14" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BC14" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BD14" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BE14" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BF14" s="5">
         <v>0</v>
@@ -4302,70 +3872,40 @@
       <c r="BK14" s="5">
         <v>0</v>
       </c>
-      <c r="BL14" s="5">
-        <v>1</v>
-      </c>
-      <c r="BM14" s="5">
-        <v>1</v>
-      </c>
-      <c r="BN14" s="5">
-        <v>1</v>
-      </c>
-      <c r="BO14" s="5">
-        <v>1</v>
-      </c>
-      <c r="BP14" s="5">
-        <v>0</v>
-      </c>
-      <c r="BQ14" s="5">
-        <v>0</v>
-      </c>
-      <c r="BR14" s="5">
-        <v>0</v>
-      </c>
-      <c r="BS14" s="5">
-        <v>0</v>
-      </c>
-      <c r="BT14" s="5">
-        <v>0</v>
-      </c>
-      <c r="BU14" s="5">
-        <v>0</v>
-      </c>
     </row>
-    <row r="15" spans="1:73" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>69</v>
       </c>
       <c r="B15" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C15" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F15" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G15" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H15" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I15" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J15" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L15" s="5">
         <v>0</v>
@@ -4506,56 +4046,26 @@
         <v>0</v>
       </c>
       <c r="BF15" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG15" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BH15" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BI15" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BJ15" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BK15" s="5">
-        <v>0</v>
-      </c>
-      <c r="BL15" s="5">
-        <v>0</v>
-      </c>
-      <c r="BM15" s="5">
-        <v>0</v>
-      </c>
-      <c r="BN15" s="5">
-        <v>0</v>
-      </c>
-      <c r="BO15" s="5">
-        <v>0</v>
-      </c>
-      <c r="BP15" s="5">
-        <v>1</v>
-      </c>
-      <c r="BQ15" s="5">
-        <v>1</v>
-      </c>
-      <c r="BR15" s="5">
-        <v>1</v>
-      </c>
-      <c r="BS15" s="5">
-        <v>1</v>
-      </c>
-      <c r="BT15" s="5">
-        <v>1</v>
-      </c>
-      <c r="BU15" s="5">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:BU15">
+  <conditionalFormatting sqref="B2:BK15">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>1</formula>
     </cfRule>

</xml_diff>